<commit_message>
Updated source of truth (data collection methodology updated and listed)
</commit_message>
<xml_diff>
--- a/Minecraft_Redstone_Block_Index.xlsx
+++ b/Minecraft_Redstone_Block_Index.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Block Index" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Block Index'!$A$1:$Q$212</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Block Index'!$A$1:$Q$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -705,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q212"/>
+  <dimension ref="A1:Q239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1527,7 +1527,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tuff</t>
+          <t>Tuff (+ Chiseled Tuff)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Movable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2460,7 +2460,11 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Full opaque block that spreads via bone meal. In Java Edition it is destroyed and dropped when pushed by a piston (movable in Bedrock Edition).</t>
+        </is>
+      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>moss-block</t>
@@ -7223,7 +7227,11 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr"/>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Crimson and Warped are the exception — Nether "wood" (their Stems, Hyphae, and stripped variants) is not flammable and cannot be set alight, unlike all Overworld log/wood species.</t>
+        </is>
+      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t>logs-wood-all-species-incl-crimson-warped-stems-stripped-variants-all-axis-orientations</t>
@@ -7294,7 +7302,11 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr"/>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Crimson and Warped Planks are the exception — Nether wood is not flammable, unlike all Overworld plank species (Bamboo Planks &amp; Mosaic included).</t>
+        </is>
+      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t>planks-all-species-incl-bamboo-planks-bamboo-mosaic</t>
@@ -7600,7 +7612,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Saplings (all species)</t>
+          <t>Saplings (all species, incl. Mangrove Propagule)</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -8188,7 +8200,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Glass Pane (clear + 16 stained) / Iron Bars</t>
+          <t>Glass Pane (clear + 16 stained) / Iron Bars / Copper Bars</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -8255,7 +8267,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>Thin cross-shaped hitbox (connects visually to neighbors) but still blocks movement through the space. Needs no support — can float freely.</t>
+          <t>Thin cross-shaped hitbox (connects visually to neighbors) but still blocks movement through the space. Needs no support. Copper Bars (added 1.21.9) oxidize but share these properties.</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -8856,11 +8868,11 @@
       </c>
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>Spans the full 16px gap while closed (blocking it); swings to a thin sliver flush with the post when open, clearing the walkway.</t>
+          <t>Closed collision box is 16px long × 4px thick × 24px tall; the 4px thickness is shown here to match the convention used for doors and other thin blocks. Opening the gate removes its collision entirely.</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -8887,7 +8899,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Doors (all wood types + Iron Door)</t>
+          <t>Doors (all wood types + Iron Door + Copper Door)</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -8954,7 +8966,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Two-block-tall object (bottom &amp; top are separate block states). The bottom half needs a solid block below it — pistons break it rather than relocating it.</t>
+          <t>Two-block-tall object (bottom &amp; top are separate block states). The bottom half needs a solid block below it — pistons break it rather than relocating it. Copper Doors (openable by hand and by redstone) oxidize but share these properties.</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -8966,7 +8978,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Trapdoors (all wood types + Iron Trapdoor)</t>
+          <t>Trapdoors (all wood types + Iron Trapdoor + Copper Trapdoor)</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -9033,7 +9045,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>Attaches to the block face it's mounted against.</t>
+          <t>Attaches to the block face it's mounted against. Copper Trapdoors oxidize but share these properties.</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
@@ -9645,7 +9657,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Pressure Plates (all wood types, Stone, Heavy Weighted/Iron, Light Weighted/Gold)</t>
+          <t>Pressure Plates (all wood types, Stone, Polished Blackstone, Heavy Weighted/Iron, Light Weighted/Gold)</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -11666,7 +11678,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Bamboo (+ Bamboo Sapling)</t>
+          <t>Bamboo (+ Bamboo Sapling, Bamboo Shoot)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -11793,11 +11805,11 @@
       </c>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>15×15×15px collision box, inset 1px from a full block on every side.</t>
+          <t>14×15×14px collision box, inset 1px from a full block on all four sides (same 14px footprint as a Honey Block).</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -13196,7 +13208,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Movable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -13247,7 +13259,11 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="P169" t="inlineStr"/>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>In Java Edition, Pumpkins / Carved Pumpkins / Jack o'Lanterns break and drop when pushed by a piston (the mechanic piston pumpkin/melon farms rely on); movable in Bedrock.</t>
+        </is>
+      </c>
       <c r="Q169" t="inlineStr">
         <is>
           <t>pumpkin-carved-pumpkin-jack-o-lantern</t>
@@ -13267,7 +13283,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Movable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -13318,7 +13334,11 @@
           <t>FALSE</t>
         </is>
       </c>
-      <c r="P170" t="inlineStr"/>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>In Java Edition, a Melon breaks and drops when pushed by a piston; movable in Bedrock.</t>
+        </is>
+      </c>
       <c r="Q170" t="inlineStr">
         <is>
           <t>melon</t>
@@ -13478,7 +13498,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Chain</t>
+          <t>Chain (Iron + Copper, all oxidation stages)</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -13545,7 +13565,7 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>Thin vertical connector block; unlike a Lantern, it can float freely without support. Thin ~2px link, nowhere near a full top face.</t>
+          <t>Thin vertical connector; unlike a Lantern it can float freely without support. Renamed from 'chain' to 'iron_chain' in 1.21.9, which also added the oxidizing Copper Chain (same properties). Thin ~3px link, nowhere near a full top face.</t>
         </is>
       </c>
       <c r="Q173" t="inlineStr">
@@ -13796,7 +13816,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Movable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -13849,7 +13869,7 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>Gravity-affected, but only falls once more than 6 blocks (through connected scaffolding) from the nearest anchoring block. Players can descend through it by holding crouch.</t>
+          <t>Gravity-affected, but only falls once more than 6 blocks (through connected scaffolding) from the nearest anchor. Breaks and drops when pushed by a piston unless it is in a falling state. Players can descend by holding crouch.</t>
         </is>
       </c>
       <c r="Q177" t="inlineStr">
@@ -14029,7 +14049,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Immovable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -14082,7 +14102,7 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>Two-block object (head + foot). Blocks piston extension entirely (stores owner/occupied state) like a chest. Explodes if used in the Nether or End. Low-profile mattress + leg shape, not a flat full-height top.</t>
+          <t>Two-block object (head + foot). Breaks and drops when pushed by a piston. Explodes if used in the Nether or End. Low-profile mattress + leg shape, not a flat full-height top.</t>
         </is>
       </c>
       <c r="Q180" t="inlineStr">
@@ -14416,7 +14436,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Immovable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -14473,7 +14493,7 @@
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>Holds a single item (tile entity) — blocks piston extension entirely. Shatters when hit by a projectile. Full-height collision box despite the visible open neck opening at the top.</t>
+          <t>Holds a single item (block entity). Breaks and drops when pushed by a piston, and shatters into sherds when hit by a projectile. Full-height collision box despite the open neck at the top.</t>
         </is>
       </c>
       <c r="Q185" t="inlineStr">
@@ -15332,7 +15352,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Immovable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -15389,7 +15409,7 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>Mounted on a floor, wall (single/double), or ceiling — needs that attachment. Blocks piston extension entirely. Bell hangs within an open frame, not a flat full top.</t>
+          <t>Mounted on a floor, wall (single/double), or ceiling. Breaks and drops when pushed by a piston. Bell hangs within an open frame, not a flat full top.</t>
         </is>
       </c>
       <c r="Q197" t="inlineStr">
@@ -15401,7 +15421,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Lantern (+ Soul Lantern)</t>
+          <t>Lantern (+ Soul Lantern, Copper Lantern)</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -15411,7 +15431,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Immovable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -15472,7 +15492,7 @@
       </c>
       <c r="P198" t="inlineStr">
         <is>
-          <t>Hangs from a block above, or sits on a block below. Blocks piston extension entirely. Open cage shape, not a flat full top.</t>
+          <t>Hangs from a block above, or sits on a block below. Breaks and drops when pushed by a piston. Open cage shape, not a flat full top. Copper Lantern (added 1.21.9) oxidizes but shares these properties.</t>
         </is>
       </c>
       <c r="Q198" t="inlineStr">
@@ -15861,7 +15881,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Immovable</t>
+          <t>Breaks</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -15914,7 +15934,7 @@
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>No collision; used as an 'eraser' inside structure templates.</t>
+          <t>No collision; used as an 'eraser' inside structure templates. Breaks when pushed by a piston in Java Edition.</t>
         </is>
       </c>
       <c r="Q204" t="inlineStr">
@@ -16515,8 +16535,2069 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Sandstone / Red Sandstone (+ Chiseled, Cut, Smooth)</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Stone &amp; Mineral</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J213" t="n">
+        <v>16</v>
+      </c>
+      <c r="K213" t="inlineStr"/>
+      <c r="L213" t="n">
+        <v>16</v>
+      </c>
+      <c r="M213" t="inlineStr"/>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Full opaque building blocks; both colors and all Chiseled/Cut/Smooth variants share these properties.</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>sandstone-red-sandstone-chiseled-cut-smooth</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Bricks</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Stone &amp; Mineral</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J214" t="n">
+        <v>16</v>
+      </c>
+      <c r="K214" t="inlineStr"/>
+      <c r="L214" t="n">
+        <v>16</v>
+      </c>
+      <c r="M214" t="inlineStr"/>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>The plain clay Bricks block (crafted from four Brick items).</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>bricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Infested Blocks (Stone, Cobblestone, Stone Bricks +Mossy/Cracked/Chiseled, Deepslate)</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Stone &amp; Mineral</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J215" t="n">
+        <v>16</v>
+      </c>
+      <c r="K215" t="inlineStr"/>
+      <c r="L215" t="n">
+        <v>16</v>
+      </c>
+      <c r="M215" t="inlineStr"/>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Identical to their host block for these properties, but release a Silverfish when broken and are mined much faster. Cannot be obtained with Silk Touch.</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>infested-blocks-stone-cobblestone-stone-bricks-mossy-cracked-chiseled-deepslate</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Pale Moss Block</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Stone &amp; Mineral</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J216" t="n">
+        <v>16</v>
+      </c>
+      <c r="K216" t="inlineStr"/>
+      <c r="L216" t="n">
+        <v>16</v>
+      </c>
+      <c r="M216" t="inlineStr"/>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Full opaque block (Pale Garden). Like Moss Block, it breaks and drops when pushed by a piston in Java Edition (movable in Bedrock).</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>pale-moss-block</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Muddy Mangrove Roots</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Dirt &amp; Organic Terrain</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J217" t="n">
+        <v>16</v>
+      </c>
+      <c r="K217" t="inlineStr"/>
+      <c r="L217" t="n">
+        <v>16</v>
+      </c>
+      <c r="M217" t="inlineStr"/>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Full opaque block, unlike the non-opaque Mangrove Roots it is crafted from.</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>muddy-mangrove-roots</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Mangrove Roots</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J218" t="n">
+        <v>16</v>
+      </c>
+      <c r="K218" t="inlineStr"/>
+      <c r="L218" t="n">
+        <v>16</v>
+      </c>
+      <c r="M218" t="inlineStr"/>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>A full cube but non-opaque (doesn't suffocate mobs), so it's not a valid spawn surface and doesn't conduct redstone. Can be waterlogged despite being a full block; flammable.</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>mangrove-roots</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Shelf (all wood types)</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Immovable</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J219" t="n">
+        <v>16</v>
+      </c>
+      <c r="K219" t="inlineStr"/>
+      <c r="L219" t="n">
+        <v>5</v>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Wall-mounted panel — 16px wide and tall but only 5px deep.</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>Stores up to 3 item stacks (block entity) — blocks piston extension entirely, like a chest. When powered by redstone, interacting swaps the shelf's contents with the player's hotbar; adjacent powered shelves connect. Added in 1.21.9 (The Copper Age). Crimson and Warped Shelves are the exception — Nether wood is not flammable.</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>shelf-all-wood-types</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Tinted Glass</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Dyed Blocks</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J220" t="n">
+        <v>16</v>
+      </c>
+      <c r="K220" t="inlineStr"/>
+      <c r="L220" t="n">
+        <v>16</v>
+      </c>
+      <c r="M220" t="inlineStr"/>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>Full cube that blocks ALL light (unlike regular Glass) yet is still non-opaque for spawning/redstone — mobs can't spawn on it and it doesn't conduct.</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>tinted-glass</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Copper Golem Statue (all oxidation stages, waxed)</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J221" t="n">
+        <v>14</v>
+      </c>
+      <c r="K221" t="inlineStr"/>
+      <c r="L221" t="n">
+        <v>10</v>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Statue shape ~10×14×10px, not a full cube.</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>Decorative poseable statue — cycles through 4 poses when used. Breaks and drops when pushed by a piston; doesn't stick to slime/honey. Oxidizes over time and can be waxed. Added in 1.21.9.</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>copper-golem-statue-all-oxidation-stages-waxed</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Dried Kelp Block</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Ocean &amp; Aquatic</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J222" t="n">
+        <v>16</v>
+      </c>
+      <c r="K222" t="inlineStr"/>
+      <c r="L222" t="n">
+        <v>16</v>
+      </c>
+      <c r="M222" t="inlineStr"/>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>Full opaque block; flammable (burns away) and usable as furnace fuel.</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>dried-kelp-block</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Hay Block</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J223" t="n">
+        <v>16</v>
+      </c>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="n">
+        <v>16</v>
+      </c>
+      <c r="M223" t="inlineStr"/>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>Full opaque block; reduces fall damage for entities landing on it. Flammable. Rotatable pillar (axis states).</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>hay-block</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Honeycomb Block</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J224" t="n">
+        <v>16</v>
+      </c>
+      <c r="K224" t="inlineStr"/>
+      <c r="L224" t="n">
+        <v>16</v>
+      </c>
+      <c r="M224" t="inlineStr"/>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>Full opaque decorative block; not flammable despite being made of honeycomb.</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>honeycomb-block</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Froglight (Ochre, Verdant, Pearlescent)</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J225" t="n">
+        <v>16</v>
+      </c>
+      <c r="K225" t="inlineStr"/>
+      <c r="L225" t="n">
+        <v>16</v>
+      </c>
+      <c r="M225" t="inlineStr"/>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>Full opaque light-emitting block (light level 15). Unlike Glowstone/Sea Lantern it IS opaque, so it conducts redstone and counts as a spawn surface.</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>froglight-ochre-verdant-pearlescent</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Shulker Box (uncolored + 16 colors)</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J226" t="n">
+        <v>16</v>
+      </c>
+      <c r="K226" t="inlineStr"/>
+      <c r="L226" t="n">
+        <v>16</v>
+      </c>
+      <c r="M226" t="inlineStr"/>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>Portable storage that keeps its contents when broken. A full cube but non-opaque (no spawns on top, non-conductive). Breaks and drops as an item when pushed by a piston; cannot be pulled. Opening needs ~half a block of clearance above its top face.</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>shulker-box-uncolored-16-colors</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Copper Chest (all oxidation stages, waxed)</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Functional Blocks (Immovable)</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Immovable</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J227" t="n">
+        <v>14</v>
+      </c>
+      <c r="K227" t="inlineStr"/>
+      <c r="L227" t="n">
+        <v>14</v>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>14×14×14px cube, inset ~1px on every side (like a regular Chest).</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>Stores items (block entity) — blocks piston extension entirely. Two placed side by side form a large copper chest. Oxidizes over time and can be waxed. Added in 1.21.9.</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>copper-chest-all-oxidation-stages-waxed</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Heavy Core</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J228" t="n">
+        <v>8</v>
+      </c>
+      <c r="K228" t="inlineStr"/>
+      <c r="L228" t="n">
+        <v>8</v>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>Small 8×8×8px core centered in the block, like a Conduit.</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>Very high blast resistance; used to craft the Mace. Movable by pistons but does not stick to slime/honey blocks.</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>heavy-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Sniffer Egg</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J229" t="n">
+        <v>16</v>
+      </c>
+      <c r="K229" t="inlineStr"/>
+      <c r="L229" t="n">
+        <v>12</v>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>~12–14px footprint, full 16px tall.</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>Hatches into a Sniffer over time (faster on Moss Block). Breaks and drops when pushed by a piston.</t>
+        </is>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>sniffer-egg</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Dried Ghast</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J230" t="n">
+        <v>10</v>
+      </c>
+      <c r="K230" t="inlineStr"/>
+      <c r="L230" t="n">
+        <v>10</v>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>~10×10×10px block, not a full cube.</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>Rehydrates in water over four stages and eventually spawns a Happy Ghast. Waterloggable. Added in 1.21.6.</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>dried-ghast</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Lightning Rod (all oxidation stages, waxed)</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Redstone Components</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Movable</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J231" t="n">
+        <v>16</v>
+      </c>
+      <c r="K231" t="inlineStr"/>
+      <c r="L231" t="n">
+        <v>4</v>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>Thin 4×4px rod spanning the full 16px height along its axis.</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>Emits a redstone signal when struck by lightning and attracts nearby strikes. Attaches to a block face; waterloggable. Oxidizes (as of 1.21.9) and can be waxed.</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>lightning-rod-all-oxidation-stages-waxed</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Cocoa (Cocoa Pods)</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J232" t="n">
+        <v>5</v>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>Grows with age: ~5px tall (age 0) up to ~9px at full growth.</t>
+        </is>
+      </c>
+      <c r="L232" t="n">
+        <v>4</v>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>Footprint grows from ~4px to ~6px with age.</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>Grows on the side of Jungle Logs/Wood through three stages. Has a small real collision box.</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>cocoa-cocoa-pods</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Spore Blossom</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" t="inlineStr"/>
+      <c r="L233" t="n">
+        <v>0</v>
+      </c>
+      <c r="M233" t="inlineStr"/>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>Hangs from a solid block above; drips water particles. No collision.</t>
+        </is>
+      </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>spore-blossom</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Pale Hanging Moss</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234" t="inlineStr"/>
+      <c r="L234" t="n">
+        <v>0</v>
+      </c>
+      <c r="M234" t="inlineStr"/>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>Hangs beneath Pale Moss Block / other blocks above (Pale Garden). No collision.</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>pale-hanging-moss</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Nether Sprouts</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K235" t="inlineStr"/>
+      <c r="L235" t="n">
+        <v>0</v>
+      </c>
+      <c r="M235" t="inlineStr"/>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>Small decorative Nether plant; needs Nylium/Soul Soil-type block below. No collision.</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>nether-sprouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Ground Cover (Pink Petals, Wildflowers, Leaf Litter)</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J236" t="n">
+        <v>0</v>
+      </c>
+      <c r="K236" t="inlineStr"/>
+      <c r="L236" t="n">
+        <v>0</v>
+      </c>
+      <c r="M236" t="inlineStr"/>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>Flat 1–4 segment ground cover that needs a solid block below. No collision. Pink Petals (Cherry Grove); Wildflowers &amp; Leaf Litter (Spring to Life).</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>ground-cover-pink-petals-wildflowers-leaf-litter</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Dry Vegetation (Bush, Firefly Bush, Short &amp; Tall Dry Grass)</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J237" t="n">
+        <v>0</v>
+      </c>
+      <c r="K237" t="inlineStr"/>
+      <c r="L237" t="n">
+        <v>0</v>
+      </c>
+      <c r="M237" t="inlineStr"/>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>Decorative dry vegetation (Spring to Life / badlands). Firefly Bush emits firefly particles at night. No collision.</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>dry-vegetation-bush-firefly-bush-short-tall-dry-grass</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Cactus Flower</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Plants &amp; Crops</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238" t="inlineStr"/>
+      <c r="L238" t="n">
+        <v>0</v>
+      </c>
+      <c r="M238" t="inlineStr"/>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>Small flower that grows on top of / beside Cactus (Spring to Life). No collision.</t>
+        </is>
+      </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>cactus-flower</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Torch / Soul Torch / Copper Torch (+ wall variants)</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Functional Blocks</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Breaks</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" t="inlineStr"/>
+      <c r="L239" t="n">
+        <v>0</v>
+      </c>
+      <c r="M239" t="inlineStr"/>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>Light source that attaches to the top or side of a block; no collision and washed away by water. Copper Torch added in 1.21.9. (The Redstone Torch is listed separately.)</t>
+        </is>
+      </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>torch-soul-torch-copper-torch-wall-variants</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q212"/>
+  <autoFilter ref="A1:Q239"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>